<commit_message>
Clean visual pass to bestseller standard + framed gallery images
Kill the boxed-grid look across all eight workbooks: cell borders become
soft bottom rules only, table headers become white-ground colored text
with a strong accent rule, KPI cards go borderless with larger numbers.
Whitespace now does the separating. Add a marketing gallery layer:
every listing screenshot wrapped in a browser-mockup frame with rounded
corners and soft shadow on a product-hue gradient (listings/gallery/,
18 images); listings now point at the framed versions. All workbooks
recalculate clean with values and insight sentences spot-verified;
screenshots and all five scored tour videos regenerated.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014AkUe8kkZr9XS2EdNVryQd
</commit_message>
<xml_diff>
--- a/products/free-simple-budget-starter.xlsx
+++ b/products/free-simple-budget-starter.xlsx
@@ -248,7 +248,7 @@
     </font>
     <font>
       <b val="true"/>
-      <sz val="16"/>
+      <sz val="18"/>
       <color rgb="FF14634C"/>
       <name val="Calibri"/>
       <family val="0"/>
@@ -256,8 +256,8 @@
     </font>
     <font>
       <b val="true"/>
-      <sz val="10"/>
-      <color rgb="FFFFFFFF"/>
+      <sz val="9"/>
+      <color rgb="FF14634C"/>
       <name val="Calibri"/>
       <family val="0"/>
       <charset val="1"/>
@@ -347,32 +347,20 @@
       <diagonal/>
     </border>
     <border diagonalUp="false" diagonalDown="false">
-      <left style="thin">
-        <color rgb="FFD8DEE9"/>
-      </left>
-      <right style="thin">
-        <color rgb="FFD8DEE9"/>
-      </right>
-      <top style="thin">
-        <color rgb="FFD8DEE9"/>
-      </top>
+      <left/>
+      <right/>
+      <top/>
       <bottom style="thin">
-        <color rgb="FFD8DEE9"/>
+        <color rgb="FFE7EBEE"/>
       </bottom>
       <diagonal/>
     </border>
     <border diagonalUp="false" diagonalDown="false">
-      <left style="thin">
-        <color rgb="FFE3E8F0"/>
-      </left>
-      <right style="thin">
-        <color rgb="FFE3E8F0"/>
-      </right>
-      <top style="thin">
-        <color rgb="FFE3E8F0"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FFE3E8F0"/>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color rgb="FF14634C"/>
       </bottom>
       <diagonal/>
     </border>
@@ -460,7 +448,7 @@
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="12" fillId="6" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="12" fillId="6" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="1" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -468,11 +456,11 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="false" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="13" fillId="6" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="13" fillId="6" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="1" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="14" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="14" fillId="6" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -546,11 +534,11 @@
       <rgbColor rgb="FF9999FF"/>
       <rgbColor rgb="FF993366"/>
       <rgbColor rgb="FFFFF6DE"/>
-      <rgbColor rgb="FFE3E8F0"/>
+      <rgbColor rgb="FFE7EBEE"/>
       <rgbColor rgb="FF660066"/>
       <rgbColor rgb="FFFF8080"/>
       <rgbColor rgb="FF0066CC"/>
-      <rgbColor rgb="FFD8DEE9"/>
+      <rgbColor rgb="FFF4F6FA"/>
       <rgbColor rgb="FF000080"/>
       <rgbColor rgb="FFFF00FF"/>
       <rgbColor rgb="FFFFFF00"/>
@@ -566,7 +554,7 @@
       <rgbColor rgb="FF99CCFF"/>
       <rgbColor rgb="FFFF99CC"/>
       <rgbColor rgb="FFCC99FF"/>
-      <rgbColor rgb="FFF4F6FA"/>
+      <rgbColor rgb="FFFFCC99"/>
       <rgbColor rgb="FF3366FF"/>
       <rgbColor rgb="FF33CCCC"/>
       <rgbColor rgb="FF99CC00"/>
@@ -911,11 +899,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="1205895"/>
-        <c:axId val="31863839"/>
+        <c:axId val="15056826"/>
+        <c:axId val="10798916"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="1205895"/>
+        <c:axId val="15056826"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -947,7 +935,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="31863839"/>
+        <c:crossAx val="10798916"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -955,7 +943,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="31863839"/>
+        <c:axId val="10798916"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -997,7 +985,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="1205895"/>
+        <c:crossAx val="15056826"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -1059,7 +1047,7 @@
       <xdr:col>10</xdr:col>
       <xdr:colOff>552600</xdr:colOff>
       <xdr:row>24</xdr:row>
-      <xdr:rowOff>149760</xdr:rowOff>
+      <xdr:rowOff>121320</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
@@ -1067,7 +1055,7 @@
         <xdr:cNvGraphicFramePr/>
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
-        <a:off x="5779800" y="1495440"/>
+        <a:off x="5779800" y="1571760"/>
         <a:ext cx="4499640" cy="3959640"/>
       </xdr:xfrm>
       <a:graphic>
@@ -1764,7 +1752,7 @@
       <c r="K3" s="2"/>
       <c r="L3" s="2"/>
     </row>
-    <row r="4" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="4" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="2"/>
       <c r="B4" s="2"/>
       <c r="C4" s="2"/>
@@ -1780,7 +1768,7 @@
       <c r="K4" s="2"/>
       <c r="L4" s="2"/>
     </row>
-    <row r="5" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="5" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="8" t="s">
         <v>18</v>
       </c>
@@ -1815,7 +1803,7 @@
       <c r="K6" s="2"/>
       <c r="L6" s="2"/>
     </row>
-    <row r="7" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="7" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="15" t="s">
         <v>19</v>
       </c>
@@ -2371,7 +2359,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{AD195614-C5D8-409E-92EF-D395FBCCD715}</x14:id>
+          <x14:id>{A05EA488-2255-4815-8FD1-B319142CAAD1}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -2388,7 +2376,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{AD195614-C5D8-409E-92EF-D395FBCCD715}">
+          <x14:cfRule type="dataBar" id="{A05EA488-2255-4815-8FD1-B319142CAAD1}">
             <x14:dataBar minLength="10" maxLength="90" axisPosition="none" gradient="true">
               <x14:cfvo type="num">
                 <xm:f>0</xm:f>

</xml_diff>